<commit_message>
Actualizacion automatica de datos desde el Boton Magico
</commit_message>
<xml_diff>
--- a/data/EVALUACIONES/AEROBICO/AEROBICO_5MIN.xlsx
+++ b/data/EVALUACIONES/AEROBICO/AEROBICO_5MIN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\ADARVE JUV D.H\App_Rendimiento_Futbol\data\EVALUACIONES\AEROBICO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AC753C1-2DA3-4CB5-A872-FA19813BE635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8422E25-C811-4801-91DF-BD818333A64D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22500" yWindow="1590" windowWidth="17280" windowHeight="9960" xr2:uid="{BBC13A56-B43E-4445-9420-3EF783FE99BE}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{BBC13A56-B43E-4445-9420-3EF783FE99BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="33">
   <si>
     <t>Fecha</t>
   </si>
@@ -220,8 +220,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{47DCDBC4-934F-4BB8-8403-1163E6A946CF}" name="Tabla1" displayName="Tabla1" ref="A1:E53" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:E53" xr:uid="{F24D9BFF-4F02-4AC6-9C99-CC9D7330899E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{47DCDBC4-934F-4BB8-8403-1163E6A946CF}" name="Tabla1" displayName="Tabla1" ref="A1:E54" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:E54" xr:uid="{F24D9BFF-4F02-4AC6-9C99-CC9D7330899E}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{B90CC2EA-DED7-4B50-9C01-6648707B7686}" name="Fecha" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{49BFBD1B-88C4-49EF-ACC0-907CF6D29923}" name="Nombre"/>
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FF0B100-72AE-4E6A-8897-D79B621AF892}">
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="28.5546875" bestFit="1" customWidth="1"/>
@@ -568,7 +568,8 @@
         <v>5</v>
       </c>
       <c r="E2" s="1">
-        <v>16.079999999999998</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>16.080000000000002</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -585,6 +586,7 @@
         <v>5</v>
       </c>
       <c r="E3" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>16.559999999999999</v>
       </c>
     </row>
@@ -602,6 +604,7 @@
         <v>5</v>
       </c>
       <c r="E4" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>16.32</v>
       </c>
     </row>
@@ -616,6 +619,7 @@
         <v>5</v>
       </c>
       <c r="E5" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>0</v>
       </c>
     </row>
@@ -633,7 +637,8 @@
         <v>5</v>
       </c>
       <c r="E6" s="1">
-        <v>17.28</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>17.279999999999998</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -650,7 +655,8 @@
         <v>5</v>
       </c>
       <c r="E7" s="1">
-        <v>16.2</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>16.200000000000003</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -667,6 +673,7 @@
         <v>5</v>
       </c>
       <c r="E8" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>17.16</v>
       </c>
     </row>
@@ -684,7 +691,8 @@
         <v>5</v>
       </c>
       <c r="E9" s="1">
-        <v>14.4</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>14.399999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -698,6 +706,7 @@
         <v>5</v>
       </c>
       <c r="E10" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>0</v>
       </c>
     </row>
@@ -715,7 +724,8 @@
         <v>5</v>
       </c>
       <c r="E11" s="1">
-        <v>16.920000000000002</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>16.919999999999998</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -732,6 +742,7 @@
         <v>5</v>
       </c>
       <c r="E12" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>16.32</v>
       </c>
     </row>
@@ -746,6 +757,7 @@
         <v>5</v>
       </c>
       <c r="E13" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>0</v>
       </c>
     </row>
@@ -763,6 +775,7 @@
         <v>5</v>
       </c>
       <c r="E14" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>15.96</v>
       </c>
     </row>
@@ -780,7 +793,8 @@
         <v>5</v>
       </c>
       <c r="E15" s="1">
-        <v>16.079999999999998</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>16.080000000000002</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -797,6 +811,7 @@
         <v>5</v>
       </c>
       <c r="E16" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>16.440000000000001</v>
       </c>
     </row>
@@ -814,6 +829,7 @@
         <v>5</v>
       </c>
       <c r="E17" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>15.96</v>
       </c>
     </row>
@@ -831,7 +847,8 @@
         <v>5</v>
       </c>
       <c r="E18" s="1">
-        <v>16.2</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>16.200000000000003</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -845,6 +862,7 @@
         <v>5</v>
       </c>
       <c r="E19" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>0</v>
       </c>
     </row>
@@ -862,7 +880,8 @@
         <v>5</v>
       </c>
       <c r="E20" s="1">
-        <v>13.8</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>13.799999999999999</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -879,6 +898,7 @@
         <v>5</v>
       </c>
       <c r="E21" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>15.72</v>
       </c>
     </row>
@@ -896,7 +916,8 @@
         <v>5</v>
       </c>
       <c r="E22" s="1">
-        <v>16.2</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>16.200000000000003</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
@@ -913,6 +934,7 @@
         <v>5</v>
       </c>
       <c r="E23" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>18</v>
       </c>
     </row>
@@ -930,7 +952,8 @@
         <v>5</v>
       </c>
       <c r="E24" s="1">
-        <v>10.32</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>10.319999999999999</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -947,7 +970,8 @@
         <v>5</v>
       </c>
       <c r="E25" s="1">
-        <v>16.8</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>16.799999999999997</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
@@ -964,6 +988,7 @@
         <v>5</v>
       </c>
       <c r="E26" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>15.96</v>
       </c>
     </row>
@@ -978,6 +1003,7 @@
         <v>5</v>
       </c>
       <c r="E27" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>0</v>
       </c>
     </row>
@@ -995,6 +1021,7 @@
         <v>5</v>
       </c>
       <c r="E28" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>14.28</v>
       </c>
     </row>
@@ -1009,6 +1036,7 @@
         <v>5</v>
       </c>
       <c r="E29" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>0</v>
       </c>
     </row>
@@ -1026,6 +1054,7 @@
         <v>5</v>
       </c>
       <c r="E30" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>16.559999999999999</v>
       </c>
     </row>
@@ -1043,7 +1072,8 @@
         <v>5</v>
       </c>
       <c r="E31" s="1">
-        <v>17.28</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>17.279999999999998</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
@@ -1060,7 +1090,8 @@
         <v>5</v>
       </c>
       <c r="E32" s="1">
-        <v>16.079999999999998</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>16.080000000000002</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
@@ -1077,6 +1108,7 @@
         <v>5</v>
       </c>
       <c r="E33" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>18.12</v>
       </c>
     </row>
@@ -1094,7 +1126,8 @@
         <v>5</v>
       </c>
       <c r="E34" s="1">
-        <v>16.2</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>16.200000000000003</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
@@ -1111,6 +1144,7 @@
         <v>5</v>
       </c>
       <c r="E35" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>18.48</v>
       </c>
     </row>
@@ -1128,6 +1162,7 @@
         <v>5</v>
       </c>
       <c r="E36" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>15</v>
       </c>
     </row>
@@ -1142,6 +1177,7 @@
         <v>5</v>
       </c>
       <c r="E37" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>0</v>
       </c>
     </row>
@@ -1159,7 +1195,8 @@
         <v>5</v>
       </c>
       <c r="E38" s="1">
-        <v>16.920000000000002</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>16.919999999999998</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
@@ -1176,7 +1213,8 @@
         <v>5</v>
       </c>
       <c r="E39" s="1">
-        <v>19.079999999999998</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>19.080000000000002</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
@@ -1190,6 +1228,7 @@
         <v>5</v>
       </c>
       <c r="E40" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>0</v>
       </c>
     </row>
@@ -1207,7 +1246,8 @@
         <v>5</v>
       </c>
       <c r="E41" s="1">
-        <v>16.2</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>16.200000000000003</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
@@ -1224,7 +1264,8 @@
         <v>5</v>
       </c>
       <c r="E42" s="1">
-        <v>16.079999999999998</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>16.080000000000002</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
@@ -1241,7 +1282,8 @@
         <v>5</v>
       </c>
       <c r="E43" s="1">
-        <v>17.760000000000002</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>17.759999999999998</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
@@ -1258,7 +1300,8 @@
         <v>5</v>
       </c>
       <c r="E44" s="1">
-        <v>15.6</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>15.600000000000001</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
@@ -1275,7 +1318,8 @@
         <v>5</v>
       </c>
       <c r="E45" s="1">
-        <v>14.88</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>14.879999999999999</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
@@ -1289,6 +1333,7 @@
         <v>5</v>
       </c>
       <c r="E46" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>0</v>
       </c>
     </row>
@@ -1306,6 +1351,7 @@
         <v>5</v>
       </c>
       <c r="E47" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>15.96</v>
       </c>
     </row>
@@ -1323,6 +1369,7 @@
         <v>5</v>
       </c>
       <c r="E48" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>16.68</v>
       </c>
     </row>
@@ -1340,6 +1387,7 @@
         <v>5</v>
       </c>
       <c r="E49" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>17.04</v>
       </c>
     </row>
@@ -1357,6 +1405,7 @@
         <v>5</v>
       </c>
       <c r="E50" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>18</v>
       </c>
     </row>
@@ -1374,7 +1423,8 @@
         <v>5</v>
       </c>
       <c r="E51" s="1">
-        <v>14.88</v>
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>14.879999999999999</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
@@ -1391,6 +1441,7 @@
         <v>5</v>
       </c>
       <c r="E52" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>17.64</v>
       </c>
     </row>
@@ -1408,7 +1459,26 @@
         <v>5</v>
       </c>
       <c r="E53" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>17.399999999999999</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54" s="2">
+        <v>46602</v>
+      </c>
+      <c r="B54" t="s">
+        <v>28</v>
+      </c>
+      <c r="C54">
+        <v>1.29</v>
+      </c>
+      <c r="D54">
+        <v>5</v>
+      </c>
+      <c r="E54" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>15.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>